<commit_message>
tested RoBERTa on sst2
</commit_message>
<xml_diff>
--- a/clairett_sentiment_data_head500.xlsx
+++ b/clairett_sentiment_data_head500.xlsx
@@ -419,12 +419,12 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
           <t>label</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>text</t>
         </is>
       </c>
     </row>

</xml_diff>